<commit_message>
Leads: 2026-10-18 01:22 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://www.rushplumbingutah.com/locations/west-jordan/sewer-line-repair</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>service@rushplumbingutah.com</t>
@@ -554,6 +553,66 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Chicago, IL | 24/7 Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>speedyplumbingchicago.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://speedyplumbingchicago.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Emergency Response</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>info@speedyplumbingchicago.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(872) 266-4670</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>emergency plumber Chicago IL</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 01:23 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -618,6 +618,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dean's Home Services</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>calldeans.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://calldeans.com/brooklyn-park/air-conditioner/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Twin Cities</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>customercare@calldeans.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>763-515-7881</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>AC installation Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 01:28 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,62 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Latty's General Plumbing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>lattysplumbing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>http://www.lattysplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@lattysplumbing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(718) 379 9356</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>76</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>plumber Bronx NY</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 01:31 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -699,7 +699,6 @@
           <t>http://www.lattysplumbing.com/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>info@lattysplumbing.com</t>
@@ -729,6 +728,62 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bellingham Trenchless Solutions</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>bellinghamtrenchlesssolutions.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://bellinghamtrenchlesssolutions.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>office@bellinghamtrenchlesssolutions.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(360) 303-5178</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>94</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>sewer repair Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 01:32 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -754,7 +754,6 @@
           <t>https://bellinghamtrenchlesssolutions.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>office@bellinghamtrenchlesssolutions.com</t>
@@ -784,6 +783,62 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Milton Frank Plumbing &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>miltonfrankplumbing.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.miltonfrankplumbing.com/residential/sewer-repairs/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@miltonfrankplumbing.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>281-645-9596</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>sewer repair The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 01:34 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -809,7 +809,6 @@
           <t>https://www.miltonfrankplumbing.com/residential/sewer-repairs/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>info@miltonfrankplumbing.com</t>
@@ -839,6 +838,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Protect Preserve Roofing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>protectpreserveroofing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://protectpreserveroofing.com/roofing-company-lakeland/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Certified Roofing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>contact@protectpreserveroofing.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(833) 777-6634</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>residential roofing company Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 01:35 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -903,6 +903,126 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Revive Roofing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>reviveroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://reviveroofingllc.com/roofing/roof-installation-services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Revive Roofing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>contact@reviveroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(614) 319-3136</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Columbus OH</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Columbus OH</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Local Furnace Repair Pro</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>localfurnacerepairpro.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://localfurnacerepairpro.com/louisiana/metairie/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Testimonials What</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>service@localfurnacerepairpro.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(877) 719-1221</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Metairie LA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>82</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>furnace repair Metairie LA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 01:37 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1023,6 +1023,62 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CMA Mechanical Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>cmahvac.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://cmahvac.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>jess.andrews@cmahvac.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(704) 784-1209</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>HVAC contractor Concord NC</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:21 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1044,7 +1044,6 @@
           <t>https://cmahvac.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>jess.andrews@cmahvac.com</t>
@@ -1074,6 +1073,62 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Baity Plumbing Company |</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>baityplumbing.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://baityplumbing.com/service-areas/winston-salem-nc/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>tdbaityplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>336-475-0921</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>plumbing company Winston Salem NC</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:23 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1099,7 +1099,6 @@
           <t>https://baityplumbing.com/service-areas/winston-salem-nc/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>tdbaityplumbing@gmail.com</t>
@@ -1129,6 +1128,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Roof Repair in Trenton, NJ | Same-Day Service</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>roofingtrentonnj.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://roofingtrentonnj.com/services/roof-repair</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Mike Rossi</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@roofingtrentonnj.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(609) 824-9079</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Trenton NJ</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>roof repair company Trenton NJ</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:25 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1193,6 +1193,126 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Thompson Electric and Air</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>thompsonelectricco.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://thompsonelectricco.com/hvac-and-ac-installation/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Follow Terms</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@thompsonelectricco.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>904-353-1500</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>AC installation Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Atlanta HVAC Contractors</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>atlantahvaccontractor.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://atlantahvaccontractor.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Founders Marcus</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@atlantahvaccontractor.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>470-847-9076</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>90</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>HVAC contractor Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:27 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1313,6 +1313,66 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>American Roofing</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>americanroofingllc.net</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://americanroofingllc.net/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>What Makes</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>americanroofingco@aol.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(315) 447-4993</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Syracuse NY</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>80</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Syracuse NY</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:31 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1373,6 +1373,66 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>All Climates Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>allclimatesheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://allclimatesheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Birmingham Hoover</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>joseph@allclimatesheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(205) 369-1070</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Birmingham AL</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>HVAC contractor Birmingham AL</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:32 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1433,6 +1433,66 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>A1 Roofing And Construction | Macon &amp; Warner Robins GA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>a1roofingmacon.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://a1roofingmacon.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>a1roofingmacon@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(478) 714-2461</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Macon GA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roofing contractor Macon GA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:34 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1493,6 +1493,118 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Miami Roofers</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>miamiroofers.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.miamiroofers.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@miamiroofers.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(305) 482-1908</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>96</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roofer Miami FL</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Roofer Orlando</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>drrooferorlando.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://drrooferorlando.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>cs@drrooferflorida.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(407) 203-9545</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>roofer Orlando FL</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:36 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1514,7 +1514,6 @@
           <t>https://www.miamiroofers.com/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>info@miamiroofers.com</t>
@@ -1570,7 +1569,6 @@
           <t>https://drrooferorlando.com/</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>cs@drrooferflorida.com</t>
@@ -1600,6 +1598,66 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Athens, GA | 24/7 Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>apexplumberathens.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://apexplumberathens.com/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Rural Clarke</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>contact@apexplumberathens.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(770) 214-4545</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Athens GA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>90</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>emergency plumber Athens GA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:44 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1663,6 +1663,62 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Plumbers | Mount Vernon, NY | Plp plumbing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>plpplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.plpplumbingheating.com/sap/plumbers/mount-vernon-ny</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>service@plpplumbingheating.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(914) 215-5412</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>plumber Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:47 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1684,7 +1684,6 @@
           <t>https://www.plpplumbingheating.com/sap/plumbers/mount-vernon-ny</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>service@plpplumbingheating.com</t>
@@ -1714,6 +1713,62 @@
         </is>
       </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Roofer Naples</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>drroofernaples.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://drroofernaples.com/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>cs@drrooferflorida.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(239) 688-5964</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roofer Naples FL</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:51 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1739,7 +1739,6 @@
           <t>https://drroofernaples.com/</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>cs@drrooferflorida.com</t>
@@ -1769,6 +1768,178 @@
         </is>
       </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Jackson  Expert Plumbing Services You Can Trust</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>jacksonplumbingerie.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.jacksonplumbingerie.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>jacksonplumbingoffice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(814) 899-1849</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Erie PA</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>plumbing company Erie PA</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Drain Cleaning in Jacksonville, FL | Aqua Breeze</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>aquabreezefl.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://aquabreezefl.com/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Aqua Breeze</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>heath@aquabreezefl.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(904) 478-5970</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>86</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>drain cleaning service Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ProTech HVAC Services</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>protech-ohio.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://protech-ohio.com/services/residential/heating/installations/heat-pumps/akron-oh</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Online Free</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>info@protech-ohio.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Akron OH</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>84</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>heat pump installation Akron OH</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 11:55 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1794,7 +1794,6 @@
           <t>https://www.jacksonplumbingerie.com/</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>jacksonplumbingoffice@gmail.com</t>
@@ -1920,7 +1919,6 @@
           <t>info@protech-ohio.com</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Akron OH</t>
@@ -1940,6 +1938,126 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Boyle Energy | Local HVAC, Oil, &amp; Propane Services</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>boylebrothersenergy.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://boylebrothersenergy.com/about-us/areas-we-serve/hvac-service-in-philadelphia/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Boyle Energy</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>info@boyleenergy.net</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>610-446-2444</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>heating and cooling company Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Water Heater Replacements &amp; Repair | Silver Spring, MD</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>khaiplumbing.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.khaiplumbing.com/water-heaters</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Leave Us</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>khaisau@gmail.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(240) 460-5041</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>88</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>water heater repair Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 12:06 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2063,6 +2063,66 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>M.S.G. Heating &amp; Air LLC</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>msgheat.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.msgheat.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Ken Hessing</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>msg.heating.air@gmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(919) 327-7196</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Raleigh NC</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>88</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>HVAC contractor Raleigh NC</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 21:26 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2123,6 +2123,62 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Rock Roofing</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>rockroofingin.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.rockroofingin.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>isaac@rockroofingin.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>260-416-4496</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>98</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>roofer Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 21:32 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2144,7 +2144,6 @@
           <t>https://www.rockroofingin.com/</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>isaac@rockroofingin.com</t>
@@ -2174,6 +2173,66 @@
         </is>
       </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Residential Roofers | Camden, NJ | Sun Roofing</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>sunroofing.biz</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.sunroofing.biz/contact/residential-roofers-service-area/camden-nj</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sun Roofing</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>roofing1@comcast.net</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(856) 784-8040</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Camden NJ</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>98</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>residential roofing company Camden NJ</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 21:34 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2238,6 +2238,66 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ListCentral.US</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>listcentral.us</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://listcentral.us/pages/directory/bangor-hvac-bangor-me</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Secure Refund</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>info@listcentral.us</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(207) 951-2028</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Bangor ME</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>HVAC contractor Bangor ME</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 21:37 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2298,6 +2298,186 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Tio Plumbing Llc</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>tioplumbing.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.tioplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Tio Plumbing</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(541) 505-4017</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Eugene OR</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>100</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>plumber Eugene OR</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Frogs Leap Solutions</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>frogsleapsolutions.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://frogsleapsolutions.com/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Junction City</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>office@frogsleapsolutions.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>541-541-5327</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Eugene OR</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>100</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>plumber Eugene OR</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tradition Plumbing</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>tradition-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://tradition-plumbing.com/eugene-or/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Tradition Plumbing</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>contact@tradition-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>541-517-7412</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Eugene OR</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>plumber Eugene OR</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 21:38 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2478,6 +2478,62 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Code Blue HVAC</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>codebluehvac.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.codebluehvac.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>info@codebluehvac.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(702) 827-1184</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>HVAC contractor North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-18 21:40 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2499,7 +2499,6 @@
           <t>https://www.codebluehvac.com/</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>info@codebluehvac.com</t>
@@ -2529,6 +2528,66 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Rooter Sewer Drain Man</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>rootersewerdrainman.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://rootersewerdrainman.com/miramar-drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>rootersewerdrainman@gmail.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>000145-2024</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>drain cleaning service Miramar FL</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-18 21:43 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-18.xlsx
+++ b/output/leads_2026-10-18.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2593,6 +2593,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Local Plumber Masters</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>localplumbermasters.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://localplumbermasters.com/delaware/newark/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Plumbing Local</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>support@localplumbermasters.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>877-388-0238</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Newark DE</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>90</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>emergency plumber Newark DE</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>